<commit_message>
Update Cargos (Permissao para ver crm engenharia(
</commit_message>
<xml_diff>
--- a/Usuarios_para_criar.xlsx
+++ b/Usuarios_para_criar.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Centauro\Meu Canto\GitHub\Centauro\CENTAURO-ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F58EBF3-57D2-4BA4-B3AA-FE719299AE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE81CE0-19EB-4B50-9873-7681560B1302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="21870" windowHeight="13050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21480" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="USER" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">USER!$A$1:$C$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="61">
   <si>
     <t>lucasdasilva@centaurotelecom.com.br</t>
   </si>
@@ -143,34 +146,82 @@
     <t>rosangela@centaurotelecom.com.br</t>
   </si>
   <si>
-    <t>reinaldo santos - sem email</t>
-  </si>
-  <si>
-    <t>jorge ramos - sem email</t>
-  </si>
-  <si>
-    <t>renato  - sem email</t>
-  </si>
-  <si>
-    <t>Assistente de Projetos</t>
-  </si>
-  <si>
-    <t>Coordenador Geral</t>
-  </si>
-  <si>
-    <t>Coordenador</t>
-  </si>
-  <si>
-    <t>Analista Comercial Pleno</t>
-  </si>
-  <si>
-    <t>Analista Comercial</t>
-  </si>
-  <si>
-    <t>Tst</t>
-  </si>
-  <si>
-    <t>Diretor</t>
+    <t>SÓCIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALISTA COMERCIAL PLENO </t>
+  </si>
+  <si>
+    <t>ASSISTENTE PROJETOS</t>
+  </si>
+  <si>
+    <t>ESTÁGIÁRIA DE ENGENHARIA</t>
+  </si>
+  <si>
+    <t>TÉCNICA DE SEGURANÇA JUNIOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALISTA DE CONTROLADORIA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">JOVEM APRENDIZ - ADMINISTRATIVO </t>
+  </si>
+  <si>
+    <t>ASSISTENTE DE RECURSOS HUMANOS</t>
+  </si>
+  <si>
+    <t>AUXILIAR ADMINISTRATIVO</t>
+  </si>
+  <si>
+    <t>ASSISTENTE FINANCEIRO</t>
+  </si>
+  <si>
+    <t>AUXILIAR FINANCEIRO</t>
+  </si>
+  <si>
+    <t>SUPERVISOR FINANCEIRO</t>
+  </si>
+  <si>
+    <t>SUPERVISOR TÉCNICO DE TELECOMUNICAÇÕES PLENO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TÉCNICO DE TELECOMUNICAÇÕES </t>
+  </si>
+  <si>
+    <t xml:space="preserve">COORDENADOR DE CONTRATOS </t>
+  </si>
+  <si>
+    <t>COORDENADOR DE TELECOMUNICAÇÕES JUNIOR</t>
+  </si>
+  <si>
+    <t>ASSISTENTE DE PROJETOS</t>
+  </si>
+  <si>
+    <t>ANALISTA ADMINISTRATIVO</t>
+  </si>
+  <si>
+    <t>ASSISTENTE COMERCIAL</t>
+  </si>
+  <si>
+    <t>ASSISTENTE FINANCEIRO SENIOR</t>
+  </si>
+  <si>
+    <t>COORDENADOR PROJETOS</t>
+  </si>
+  <si>
+    <t>1002T</t>
+  </si>
+  <si>
+    <t>1001T</t>
+  </si>
+  <si>
+    <t>1000T</t>
+  </si>
+  <si>
+    <t>DIRETOR</t>
+  </si>
+  <si>
+    <t>39T</t>
   </si>
 </sst>
 </file>
@@ -186,18 +237,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -212,16 +257,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -504,23 +542,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -531,16 +568,19 @@
       <c r="B2" s="1">
         <v>474</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>38</v>
+      <c r="C2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>39</v>
+      <c r="B3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -550,16 +590,19 @@
       <c r="B4" s="1">
         <v>375</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>40</v>
+      <c r="C4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>40</v>
+      <c r="B5" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -569,8 +612,8 @@
       <c r="B6" s="1">
         <v>339</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>41</v>
+      <c r="C6" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -580,8 +623,8 @@
       <c r="B7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>42</v>
+      <c r="C7" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -591,8 +634,8 @@
       <c r="B8" s="1">
         <v>589</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>42</v>
+      <c r="C8" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -602,8 +645,8 @@
       <c r="B9" s="1">
         <v>564</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>43</v>
+      <c r="C9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -613,7 +656,7 @@
       <c r="B10" s="1">
         <v>2073</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>38</v>
       </c>
     </row>
@@ -621,24 +664,33 @@
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>44</v>
+      <c r="B11" s="1">
+        <v>1002</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>44</v>
+      <c r="B12" s="1">
+        <v>1001</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>44</v>
+      <c r="B13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -648,6 +700,9 @@
       <c r="B14" s="1">
         <v>376</v>
       </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -656,6 +711,9 @@
       <c r="B15" s="1">
         <v>604</v>
       </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -664,145 +722,189 @@
       <c r="B16" s="1">
         <v>439</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
       <c r="B17" s="1">
         <v>575</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="1">
         <v>567</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1">
         <v>556</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="1">
         <v>608</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>3000</v>
+      </c>
+      <c r="C22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="1">
         <v>309</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="1">
         <v>548</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="1">
         <v>182</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="B26" s="1">
+        <v>526</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="B27" s="1">
+        <v>264</v>
+      </c>
+      <c r="C27" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B28" s="1">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <v>510</v>
+      </c>
+      <c r="C28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>263</v>
+      </c>
+      <c r="C29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+      <c r="C30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+      <c r="C31" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" s="1">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" s="1">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="1">
         <v>577</v>
       </c>
+      <c r="C32" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Colaboradores / Roles (Adicionei uma role para liberar todos)
</commit_message>
<xml_diff>
--- a/Usuarios_para_criar.xlsx
+++ b/Usuarios_para_criar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Centauro\Meu Canto\GitHub\Centauro\CENTAURO-ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE81CE0-19EB-4B50-9873-7681560B1302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03AD8E7-CE4E-4C42-B79C-4ACD2530E5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21480" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="50">
   <si>
     <t>lucasdasilva@centaurotelecom.com.br</t>
   </si>
@@ -155,57 +155,12 @@
     <t>ASSISTENTE PROJETOS</t>
   </si>
   <si>
-    <t>ESTÁGIÁRIA DE ENGENHARIA</t>
-  </si>
-  <si>
-    <t>TÉCNICA DE SEGURANÇA JUNIOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANALISTA DE CONTROLADORIA </t>
-  </si>
-  <si>
-    <t xml:space="preserve">JOVEM APRENDIZ - ADMINISTRATIVO </t>
-  </si>
-  <si>
-    <t>ASSISTENTE DE RECURSOS HUMANOS</t>
-  </si>
-  <si>
-    <t>AUXILIAR ADMINISTRATIVO</t>
-  </si>
-  <si>
-    <t>ASSISTENTE FINANCEIRO</t>
-  </si>
-  <si>
-    <t>AUXILIAR FINANCEIRO</t>
-  </si>
-  <si>
-    <t>SUPERVISOR FINANCEIRO</t>
-  </si>
-  <si>
-    <t>SUPERVISOR TÉCNICO DE TELECOMUNICAÇÕES PLENO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TÉCNICO DE TELECOMUNICAÇÕES </t>
-  </si>
-  <si>
-    <t xml:space="preserve">COORDENADOR DE CONTRATOS </t>
-  </si>
-  <si>
-    <t>COORDENADOR DE TELECOMUNICAÇÕES JUNIOR</t>
-  </si>
-  <si>
     <t>ASSISTENTE DE PROJETOS</t>
   </si>
   <si>
-    <t>ANALISTA ADMINISTRATIVO</t>
-  </si>
-  <si>
     <t>ASSISTENTE COMERCIAL</t>
   </si>
   <si>
-    <t>ASSISTENTE FINANCEIRO SENIOR</t>
-  </si>
-  <si>
     <t>COORDENADOR PROJETOS</t>
   </si>
   <si>
@@ -222,6 +177,18 @@
   </si>
   <si>
     <t>39T</t>
+  </si>
+  <si>
+    <t>FINANCEIRO</t>
+  </si>
+  <si>
+    <t>RH &amp; DP</t>
+  </si>
+  <si>
+    <t>CONTROLADORIA</t>
+  </si>
+  <si>
+    <t>TST</t>
   </si>
 </sst>
 </file>
@@ -237,12 +204,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -257,11 +230,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,7 +536,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1">
@@ -573,40 +547,40 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>375</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1">
@@ -617,40 +591,40 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1">
         <v>589</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1">
         <v>564</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1">
@@ -661,128 +635,128 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="1">
         <v>1002</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="1">
         <v>1001</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="1">
         <v>376</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="1">
         <v>604</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="1">
         <v>439</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B17" s="1">
         <v>575</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="1">
         <v>567</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="1">
         <v>556</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="1">
         <v>608</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="1">
@@ -793,113 +767,113 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="1">
         <v>309</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="1">
         <v>548</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="1">
         <v>182</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="1">
         <v>526</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="A27" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B27" s="1">
         <v>264</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="1">
         <v>510</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="1">
         <v>263</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="1">
         <v>149</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="1">
         <v>161</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="1">
         <v>577</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>